<commit_message>
feat(cohort): add age outlier detection for children >=60 months in period 2 and update sample data
</commit_message>
<xml_diff>
--- a/public/data/sample-stunting-periode-1.xlsx
+++ b/public/data/sample-stunting-periode-1.xlsx
@@ -397,7 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
+  <cols>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="25.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,7 +432,7 @@
         <v>Desa/Kelurahan</v>
       </c>
       <c r="H1" t="str">
-        <v>Status Stunting</v>
+        <v>Status Gizi</v>
       </c>
     </row>
     <row r="2">
@@ -482,13 +492,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>3301020301230003</v>
+        <v>3301020301210003</v>
       </c>
       <c r="C4" t="str">
-        <v>Budi Santoso</v>
+        <v>Budi Santoso (Outlier Usia)</v>
       </c>
       <c r="D4" t="str">
-        <v>2023-01-03</v>
+        <v>2021-04-10</v>
       </c>
       <c r="E4" t="str">
         <v>L</v>
@@ -690,7 +700,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>3301061912220011</v>
+        <v>3301061908210011</v>
       </c>
       <c r="C12" t="str">
         <v>Rafi Pratama</v>
@@ -711,9 +721,35 @@
         <v>Stunting</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>3301065103210012</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Salma Kirana</v>
+      </c>
+      <c r="D13" t="str">
+        <v>2021-03-15</v>
+      </c>
+      <c r="E13" t="str">
+        <v>P</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Puskesmas Gayamsari</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Pandean Lamper</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Stunting</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>